<commit_message>
오늘의 할인: DiscountCostCount 반영
할인가가 적힌 상품만 오늘의 할인 후보다. 빈 칸이면 제외 — 팽이코인이
그렇게 빠진다. 정가보다 크거나 같으면 할인으로 안 친다.

- 원가에 취소선(회색), 옆에 할인가(빨강). 취소선은 아트가 아니라 얇은
  사각형이고 글자 폭에 맞춰 런타임에 줄인다 — 칸 폭 그대로면 짧은 숫자에서
  허공까지 그어진다
- 할인가는 오늘의 할인 칸에서만 적용된다. 카테고리 목록에서는 같은 상품이라도
  정가라, 구매 이벤트에 어디서 눌렀는지를 같이 싣는다
- 할인 상품이 하나도 없으면 패널이 「준비중입니다」가 되고 구매 버튼이 숨는다

확인: 콘솔 하네스 71건. 할인 9 / 빈 칸 1, 할인 칸에서 상추를 3에 사고
목록에서는 5 를 받는 것까지.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SnailData.xlsx
+++ b/SnailData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjwog\Desktop\SnailProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0E124E-4EC3-4A0E-A06E-3E6DDA867E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BB587D7-C2B4-4A4A-9644-07D41B070B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="866" firstSheet="2" activeTab="15" xr2:uid="{5EE1C0BB-DAD6-4BF1-AA41-9BEEACC3D6EF}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="866" firstSheet="2" activeTab="11" xr2:uid="{5EE1C0BB-DAD6-4BF1-AA41-9BEEACC3D6EF}"/>
   </bookViews>
   <sheets>
     <sheet name="EnumData" sheetId="8" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="473">
   <si>
     <t>ALL</t>
   </si>
@@ -1722,6 +1722,10 @@
   </si>
   <si>
     <t>준비중입니다.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DiscountCostCount</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1924,7 +1928,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1963,6 +1967,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3349,21 +3356,21 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E79052-7558-4F08-8689-6E3AEA3B2BB4}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.125" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="17.625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.75" customWidth="1"/>
-    <col min="7" max="7" width="28.125" customWidth="1"/>
-    <col min="8" max="8" width="23.125" customWidth="1"/>
-    <col min="9" max="9" width="19.375" customWidth="1"/>
-    <col min="10" max="10" width="16.125" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="6" max="7" width="17.75" customWidth="1"/>
+    <col min="8" max="8" width="28.125" customWidth="1"/>
+    <col min="9" max="9" width="23.125" customWidth="1"/>
+    <col min="10" max="10" width="19.375" customWidth="1"/>
+    <col min="11" max="11" width="16.125" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -3389,16 +3396,19 @@
         <v>0</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="7" t="s">
-        <v>0</v>
-      </c>
       <c r="K1" s="7" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>88</v>
       </c>
@@ -3418,22 +3428,25 @@
         <v>71</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>101</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>89</v>
       </c>
@@ -3453,22 +3466,25 @@
         <v>65</v>
       </c>
       <c r="G3" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -3487,24 +3503,27 @@
       <c r="F4">
         <v>5</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="14">
+        <v>3</v>
+      </c>
+      <c r="H4" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
         <v>70</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <f>F4/2</f>
         <v>2.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -3523,24 +3542,27 @@
       <c r="F5">
         <v>7</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="14">
+        <v>4</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
         <v>70</v>
       </c>
-      <c r="K5">
-        <f t="shared" ref="K5:K9" si="0">F5/2</f>
+      <c r="L5">
+        <f t="shared" ref="L5:L9" si="0">F5/2</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -3559,24 +3581,27 @@
       <c r="F6">
         <v>7</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="14">
+        <v>4</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I6" t="b">
-        <v>0</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s">
         <v>70</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>93</v>
       </c>
@@ -3595,24 +3620,27 @@
       <c r="F7">
         <v>12</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="14">
+        <v>8</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I7" t="b">
-        <v>0</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="s">
         <v>70</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>91</v>
       </c>
@@ -3631,24 +3659,27 @@
       <c r="F8">
         <v>50</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="14">
+        <v>35</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I8" t="b">
-        <v>0</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s">
         <v>70</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>91</v>
       </c>
@@ -3667,24 +3698,27 @@
       <c r="F9">
         <v>300</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="14">
+        <v>210</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I9" t="b">
-        <v>0</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="s">
         <v>70</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <f t="shared" si="0"/>
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>97</v>
       </c>
@@ -3703,17 +3737,18 @@
       <c r="F10">
         <v>1</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="14"/>
+      <c r="H10" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="I10" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>111</v>
       </c>
@@ -3732,24 +3767,27 @@
       <c r="F11">
         <v>500</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="14">
+        <v>350</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I11" t="b">
-        <v>0</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s">
         <v>70</v>
       </c>
-      <c r="K11">
-        <f t="shared" ref="K11:K13" si="1">F11/2</f>
+      <c r="L11">
+        <f t="shared" ref="L11:L13" si="1">F11/2</f>
         <v>250</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -3768,24 +3806,27 @@
       <c r="F12">
         <v>500</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="14">
+        <v>350</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I12" t="b">
-        <v>0</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" t="s">
         <v>70</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <f t="shared" si="1"/>
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>111</v>
       </c>
@@ -3804,19 +3845,22 @@
       <c r="F13">
         <v>500</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="14">
+        <v>350</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="I13" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I13" t="b">
-        <v>0</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
+      <c r="K13" t="s">
         <v>70</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <f t="shared" si="1"/>
         <v>250</v>
       </c>

</xml_diff>